<commit_message>
updating crop acreage for september
</commit_message>
<xml_diff>
--- a/data-raw/fsaCropAcreage/fsa_acreage_urls.xlsx
+++ b/data-raw/fsaCropAcreage/fsa_acreage_urls.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10817"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10913"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dylanturner/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dylanturner/Library/CloudStorage/Dropbox/rfsa/data-raw/fsaCropAcreage/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF539E9D-6EDE-5E4A-891A-0622D3E6EA42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EF6F6A9-EF0E-CC48-B888-53ECFFB3C053}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="55280" yWindow="1120" windowWidth="25620" windowHeight="15920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="142">
   <si>
     <t>raw_string</t>
   </si>
@@ -440,6 +440,12 @@
   </si>
   <si>
     <t>2025 acreage data as of August 1, 2025</t>
+  </si>
+  <si>
+    <t>2025 acreage data as of September 12, 2025</t>
+  </si>
+  <si>
+    <t>https://www.fsa.usda.gov/sites/default/files/2025-09/AwCPYHfbDXJx.zip</t>
   </si>
 </sst>
 </file>
@@ -796,7 +802,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F71"/>
+  <dimension ref="A1:F72"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="51.5" customWidth="1"/>
@@ -2224,6 +2230,26 @@
         <v>138</v>
       </c>
     </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A72" t="s">
+        <v>140</v>
+      </c>
+      <c r="B72">
+        <v>12</v>
+      </c>
+      <c r="C72">
+        <v>9</v>
+      </c>
+      <c r="D72">
+        <v>2025</v>
+      </c>
+      <c r="E72" s="2">
+        <v>45912</v>
+      </c>
+      <c r="F72" t="s">
+        <v>141</v>
+      </c>
+    </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F69">
     <sortCondition ref="E1:E69"/>

</xml_diff>

<commit_message>
Updating fsa crop acreage data based on december release
</commit_message>
<xml_diff>
--- a/data-raw/fsaCropAcreage/fsa_acreage_urls.xlsx
+++ b/data-raw/fsaCropAcreage/fsa_acreage_urls.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10913"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11214"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dylanturner/Library/CloudStorage/Dropbox/rfsa/data-raw/fsaCropAcreage/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dylanturner/Library/CloudStorage/Dropbox-Personal/rfsa/data-raw/fsaCropAcreage/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EF6F6A9-EF0E-CC48-B888-53ECFFB3C053}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B80946D7-CFA0-E54D-A7E1-12769A203C8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="55280" yWindow="1120" windowWidth="25620" windowHeight="15920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="8420" yWindow="660" windowWidth="25620" windowHeight="15920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="144">
   <si>
     <t>raw_string</t>
   </si>
@@ -446,6 +446,12 @@
   </si>
   <si>
     <t>https://www.fsa.usda.gov/sites/default/files/2025-09/AwCPYHfbDXJx.zip</t>
+  </si>
+  <si>
+    <t>2025 acreage data as of December 9, 2025</t>
+  </si>
+  <si>
+    <t>https://www.fsa.usda.gov/sites/default/files/2025-12/UhYA3k5AKxVM.zip</t>
   </si>
 </sst>
 </file>
@@ -802,7 +808,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F72"/>
+  <dimension ref="A1:F73"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="51.5" customWidth="1"/>
@@ -2250,6 +2256,26 @@
         <v>141</v>
       </c>
     </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A73" t="s">
+        <v>142</v>
+      </c>
+      <c r="B73">
+        <v>9</v>
+      </c>
+      <c r="C73">
+        <v>12</v>
+      </c>
+      <c r="D73">
+        <v>2025</v>
+      </c>
+      <c r="E73" s="2">
+        <v>46000</v>
+      </c>
+      <c r="F73" t="s">
+        <v>143</v>
+      </c>
+    </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F69">
     <sortCondition ref="E1:E69"/>

</xml_diff>

<commit_message>
correcting wrong date in fsa_acreage_urls.xlsx
</commit_message>
<xml_diff>
--- a/data-raw/fsaCropAcreage/fsa_acreage_urls.xlsx
+++ b/data-raw/fsaCropAcreage/fsa_acreage_urls.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10208"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10322"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dylanturner/Library/CloudStorage/Dropbox-Personal/rfsa/data-raw/fsaCropAcreage/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9C9C024-12F6-0846-8D78-13E423CA7A08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD0C02B1-6A5D-9740-B84D-86585CD99B78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-19480" yWindow="-31500" windowWidth="30740" windowHeight="26600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1907,10 +1907,10 @@
         <v>18</v>
       </c>
       <c r="B55">
+        <v>1</v>
+      </c>
+      <c r="C55">
         <v>12</v>
-      </c>
-      <c r="C55">
-        <v>1</v>
       </c>
       <c r="D55">
         <v>2022</v>

</xml_diff>

<commit_message>
correcting another malformed date string
</commit_message>
<xml_diff>
--- a/data-raw/fsaCropAcreage/fsa_acreage_urls.xlsx
+++ b/data-raw/fsaCropAcreage/fsa_acreage_urls.xlsx
@@ -8,14 +8,27 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dylanturner/Library/CloudStorage/Dropbox-Personal/rfsa/data-raw/fsaCropAcreage/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD0C02B1-6A5D-9740-B84D-86585CD99B78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5808F04-942E-C644-BACE-5D0208CC6547}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10160" yWindow="1140" windowWidth="30240" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -1127,10 +1140,10 @@
         <v>90</v>
       </c>
       <c r="B16">
+        <v>1</v>
+      </c>
+      <c r="C16">
         <v>9</v>
-      </c>
-      <c r="C16">
-        <v>1</v>
       </c>
       <c r="D16">
         <v>2016</v>

</xml_diff>

<commit_message>
Updating fsa planted acreage based on august data release
</commit_message>
<xml_diff>
--- a/data-raw/fsaCropAcreage/fsa_acreage_urls.xlsx
+++ b/data-raw/fsaCropAcreage/fsa_acreage_urls.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10322"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10821"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dylanturner/Library/CloudStorage/Dropbox-Personal/rfsa/data-raw/fsaCropAcreage/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5808F04-942E-C644-BACE-5D0208CC6547}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5EE7A08-587D-444E-8B46-B3F7E4B0C43B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10160" yWindow="1140" windowWidth="30240" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="820" windowWidth="30240" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="148">
   <si>
     <t>raw_string</t>
   </si>
@@ -471,6 +471,12 @@
   </si>
   <si>
     <t>https://www.fsa.usda.gov/sites/default/files/2026-01/DoISjehvQfz9.ZIP</t>
+  </si>
+  <si>
+    <t>2026 acreage data as of August 12, 2026</t>
+  </si>
+  <si>
+    <t>https://www.fsa.usda.gov/sites/default/files/2026-08/jhIRZDbkVKX5.zip</t>
   </si>
 </sst>
 </file>
@@ -827,7 +833,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F74"/>
+  <dimension ref="A1:F75"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="51.5" customWidth="1"/>
@@ -2315,6 +2321,26 @@
         <v>145</v>
       </c>
     </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A75" t="s">
+        <v>146</v>
+      </c>
+      <c r="B75">
+        <v>12</v>
+      </c>
+      <c r="C75">
+        <v>8</v>
+      </c>
+      <c r="D75">
+        <v>2026</v>
+      </c>
+      <c r="E75" s="2">
+        <v>46246</v>
+      </c>
+      <c r="F75" t="s">
+        <v>147</v>
+      </c>
+    </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F69">
     <sortCondition ref="E1:E69"/>

</xml_diff>